<commit_message>
feat(skill): 技能数值经 sim:pacing 重校准 + 记忆同步
- 技能定位为节奏点缀：压倍率/升触发（旋风斩 10次×0.5、裂地击 8s×1.2、致命一击 15次×2.5）
- L7/L10 怪 hp ×1.4、Boss 血 15100，技能生效状态下 13 门槛复绿
- 同步项目状态/设计日志/代码地图，收录技能系统设计文档与实现计划

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/config-xlsx/battle.xlsx
+++ b/tools/config-xlsx/battle.xlsx
@@ -823,7 +823,7 @@
         <v>150,40,40</v>
       </c>
       <c r="G5">
-        <v>10800</v>
+        <v>15100</v>
       </c>
       <c r="H5">
         <v>55</v>
@@ -2043,7 +2043,7 @@
         <v>0.4</v>
       </c>
       <c r="I37">
-        <v>480</v>
+        <v>670</v>
       </c>
     </row>
     <row r="38">
@@ -2072,7 +2072,7 @@
         <v>1.2</v>
       </c>
       <c r="I38">
-        <v>1345</v>
+        <v>1885</v>
       </c>
     </row>
     <row r="39">
@@ -2101,7 +2101,7 @@
         <v>0.4</v>
       </c>
       <c r="I39">
-        <v>265</v>
+        <v>370</v>
       </c>
     </row>
     <row r="40">
@@ -2130,7 +2130,7 @@
         <v>1.2</v>
       </c>
       <c r="I40">
-        <v>1345</v>
+        <v>1885</v>
       </c>
     </row>
     <row r="41">
@@ -2159,7 +2159,7 @@
         <v>0.4</v>
       </c>
       <c r="I41">
-        <v>480</v>
+        <v>670</v>
       </c>
     </row>
     <row r="42">
@@ -2188,7 +2188,7 @@
         <v>1.4</v>
       </c>
       <c r="I42">
-        <v>1345</v>
+        <v>1885</v>
       </c>
     </row>
     <row r="43">
@@ -2217,7 +2217,7 @@
         <v>0.6</v>
       </c>
       <c r="I43">
-        <v>265</v>
+        <v>370</v>
       </c>
     </row>
     <row r="44">
@@ -2652,7 +2652,7 @@
         <v>0.35</v>
       </c>
       <c r="I58">
-        <v>575</v>
+        <v>805</v>
       </c>
     </row>
     <row r="59">
@@ -2681,7 +2681,7 @@
         <v>0.4</v>
       </c>
       <c r="I59">
-        <v>290</v>
+        <v>405</v>
       </c>
     </row>
     <row r="60">
@@ -2710,7 +2710,7 @@
         <v>1.2</v>
       </c>
       <c r="I60">
-        <v>1440</v>
+        <v>2015</v>
       </c>
     </row>
     <row r="61">
@@ -2739,7 +2739,7 @@
         <v>0.4</v>
       </c>
       <c r="I61">
-        <v>575</v>
+        <v>805</v>
       </c>
     </row>
     <row r="62">
@@ -2768,7 +2768,7 @@
         <v>0.5</v>
       </c>
       <c r="I62">
-        <v>290</v>
+        <v>405</v>
       </c>
     </row>
     <row r="63">
@@ -2826,7 +2826,7 @@
         <v>0.8</v>
       </c>
       <c r="I64">
-        <v>290</v>
+        <v>405</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(squad): squadCap 接入 battle 配置链路
Misc 加 squadCap=2，导表器组装 + BattleConfig 类型 + seed:battle 脚本。
roster 保持 dps 不变，生成产物零平衡改动。

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/config-xlsx/battle.xlsx
+++ b/tools/config-xlsx/battle.xlsx
@@ -2838,7 +2838,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2858,63 +2858,71 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>roster</v>
-      </c>
-      <c r="B3" t="str">
-        <v>dps</v>
+        <v>squadCap</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>combat.minDamageRate</v>
-      </c>
-      <c r="B4">
-        <v>0.1</v>
+        <v>roster</v>
+      </c>
+      <c r="B4" t="str">
+        <v>dps</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>layout.frontMargin</v>
+        <v>combat.minDamageRate</v>
       </c>
       <c r="B5">
-        <v>360</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>layout.spacing</v>
+        <v>layout.frontMargin</v>
       </c>
       <c r="B6">
-        <v>110</v>
+        <v>360</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>bullet.speed</v>
+        <v>layout.spacing</v>
       </c>
       <c r="B7">
-        <v>1100</v>
+        <v>110</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>bullet.radius</v>
+        <v>bullet.speed</v>
       </c>
       <c r="B8">
-        <v>8</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
+        <v>bullet.radius</v>
+      </c>
+      <c r="B9">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
         <v>formation.contactGap</v>
       </c>
-      <c r="B9">
+      <c r="B10">
         <v>150</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B10"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat(squad): pacing-sim 按组合参数化 + 默认 tank+dps 逐关重调平衡
winRate 按 roster 给每个出战角色套装备档；配置默认组合翻成 tank+dps。
双人后仅两台阶失守：L7 怪 hp ×1.15（t1 0%/t2 100%）、L10 Boss 血 15100→36000
覆盖（t2 0%/t3 100%）；13 门槛连跑 6 次全绿。
抽查：dps+healer 可玩；tank+healer 无输出 0%（设计取舍，需带输出角色）。

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/config-xlsx/battle.xlsx
+++ b/tools/config-xlsx/battle.xlsx
@@ -2043,7 +2043,7 @@
         <v>0.4</v>
       </c>
       <c r="I37">
-        <v>670</v>
+        <v>770</v>
       </c>
     </row>
     <row r="38">
@@ -2072,7 +2072,7 @@
         <v>1.2</v>
       </c>
       <c r="I38">
-        <v>1885</v>
+        <v>2168</v>
       </c>
     </row>
     <row r="39">
@@ -2101,7 +2101,7 @@
         <v>0.4</v>
       </c>
       <c r="I39">
-        <v>370</v>
+        <v>426</v>
       </c>
     </row>
     <row r="40">
@@ -2130,7 +2130,7 @@
         <v>1.2</v>
       </c>
       <c r="I40">
-        <v>1885</v>
+        <v>2168</v>
       </c>
     </row>
     <row r="41">
@@ -2159,7 +2159,7 @@
         <v>0.4</v>
       </c>
       <c r="I41">
-        <v>670</v>
+        <v>770</v>
       </c>
     </row>
     <row r="42">
@@ -2188,7 +2188,7 @@
         <v>1.4</v>
       </c>
       <c r="I42">
-        <v>1885</v>
+        <v>2168</v>
       </c>
     </row>
     <row r="43">
@@ -2217,7 +2217,7 @@
         <v>0.6</v>
       </c>
       <c r="I43">
-        <v>370</v>
+        <v>426</v>
       </c>
     </row>
     <row r="44">
@@ -2796,8 +2796,8 @@
       <c r="H63">
         <v>1</v>
       </c>
-      <c r="I63" t="str">
-        <v/>
+      <c r="I63">
+        <v>36000</v>
       </c>
     </row>
     <row r="64">
@@ -2869,7 +2869,7 @@
         <v>roster</v>
       </c>
       <c r="B4" t="str">
-        <v>dps</v>
+        <v>tank,dps</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
feat(growth): charGrowth 配置 + EnemyTypes.exp 接入 battle 配置链路
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/config-xlsx/battle.xlsx
+++ b/tools/config-xlsx/battle.xlsx
@@ -577,7 +577,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R5"/>
+  <dimension ref="A1:S5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -634,6 +634,9 @@
       <c r="R1" t="str">
         <v>dmgReduce</v>
       </c>
+      <c r="S1" t="str">
+        <v>exp</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -690,6 +693,9 @@
       <c r="R2">
         <v>0</v>
       </c>
+      <c r="S2">
+        <v>5</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -746,6 +752,9 @@
       <c r="R3">
         <v>0</v>
       </c>
+      <c r="S3">
+        <v>4</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -802,6 +811,9 @@
       <c r="R4">
         <v>0.15</v>
       </c>
+      <c r="S4">
+        <v>10</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -858,10 +870,13 @@
       <c r="R5">
         <v>0.3</v>
       </c>
+      <c r="S5">
+        <v>200</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:R5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S5"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2838,7 +2853,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B14"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2874,55 +2889,87 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>combat.minDamageRate</v>
+        <v>charGrowth.expBase</v>
       </c>
       <c r="B5">
-        <v>0.1</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>layout.frontMargin</v>
+        <v>charGrowth.expGrowthPerLevel</v>
       </c>
       <c r="B6">
-        <v>360</v>
+        <v>1.15</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>layout.spacing</v>
+        <v>charGrowth.statGrowthPerLevel</v>
       </c>
       <c r="B7">
-        <v>110</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>bullet.speed</v>
+        <v>charGrowth.maxLevel</v>
       </c>
       <c r="B8">
-        <v>1100</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>bullet.radius</v>
+        <v>combat.minDamageRate</v>
       </c>
       <c r="B9">
-        <v>8</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
+        <v>layout.frontMargin</v>
+      </c>
+      <c r="B10">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>layout.spacing</v>
+      </c>
+      <c r="B11">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>bullet.speed</v>
+      </c>
+      <c r="B12">
+        <v>1100</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>bullet.radius</v>
+      </c>
+      <c r="B13">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
         <v>formation.contactGap</v>
       </c>
-      <c r="B10">
+      <c r="B14">
         <v>150</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B14"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
refactor(战斗框架): moveSpeed 迁入 CombatStats 统一属性表——减速可 Buff 化
- CombatStats 加 moveSpeed；classes.moveSpeed/enemyTypes.speed 顶层字段废弃，数值等价搬运（tank/dps 300、healer 补 220 仅供行军、怪物原 speed 原样）
- CombatUnit 删单位字段，读取全走 stats.moveSpeed（近战冲锋/怪推进即刻吃 Buff 减速）；normalizeStats 钳非负
- ConfigPanel 统一属性行自动出移速滑块；buff.xlsx 种占位 frost 冰缓（moveSpeed%:-0.3）

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/config-xlsx/battle.xlsx
+++ b/tools/config-xlsx/battle.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:N4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -444,6 +444,9 @@
       <c r="M1" t="str">
         <v>dmgReduce</v>
       </c>
+      <c r="N1" t="str">
+        <v>moveSpeed</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -485,6 +488,9 @@
       <c r="M2">
         <v>0.1</v>
       </c>
+      <c r="N2">
+        <v>300</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -526,6 +532,9 @@
       <c r="M3">
         <v>0</v>
       </c>
+      <c r="N3">
+        <v>300</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -567,10 +576,13 @@
       <c r="M4">
         <v>0</v>
       </c>
+      <c r="N4">
+        <v>220</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N4"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -587,52 +599,52 @@
         <v>name</v>
       </c>
       <c r="C1" t="str">
-        <v>speed</v>
+        <v>radius</v>
       </c>
       <c r="D1" t="str">
-        <v>radius</v>
+        <v>attackInterval</v>
       </c>
       <c r="E1" t="str">
-        <v>attackInterval</v>
+        <v>color</v>
       </c>
       <c r="F1" t="str">
-        <v>color</v>
+        <v>hp</v>
       </c>
       <c r="G1" t="str">
-        <v>hp</v>
+        <v>atk</v>
       </c>
       <c r="H1" t="str">
-        <v>atk</v>
+        <v>def</v>
       </c>
       <c r="I1" t="str">
-        <v>def</v>
+        <v>range</v>
       </c>
       <c r="J1" t="str">
-        <v>range</v>
+        <v>attackSpeed</v>
       </c>
       <c r="K1" t="str">
-        <v>attackSpeed</v>
+        <v>critRate</v>
       </c>
       <c r="L1" t="str">
-        <v>critRate</v>
+        <v>critDmg</v>
       </c>
       <c r="M1" t="str">
-        <v>critDmg</v>
+        <v>dodgeRate</v>
       </c>
       <c r="N1" t="str">
-        <v>dodgeRate</v>
+        <v>blockRate</v>
       </c>
       <c r="O1" t="str">
-        <v>blockRate</v>
+        <v>blockRatio</v>
       </c>
       <c r="P1" t="str">
-        <v>blockRatio</v>
+        <v>dmgBonus</v>
       </c>
       <c r="Q1" t="str">
-        <v>dmgBonus</v>
+        <v>dmgReduce</v>
       </c>
       <c r="R1" t="str">
-        <v>dmgReduce</v>
+        <v>moveSpeed</v>
       </c>
       <c r="S1" t="str">
         <v>exp</v>
@@ -646,52 +658,52 @@
         <v>丧尸</v>
       </c>
       <c r="C2">
+        <v>28</v>
+      </c>
+      <c r="D2">
+        <v>0.8</v>
+      </c>
+      <c r="E2" t="str">
+        <v>230,70,70</v>
+      </c>
+      <c r="F2">
+        <v>120</v>
+      </c>
+      <c r="G2">
+        <v>18</v>
+      </c>
+      <c r="H2">
+        <v>4</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2">
+        <v>1</v>
+      </c>
+      <c r="K2">
+        <v>0.05</v>
+      </c>
+      <c r="L2">
+        <v>0.5</v>
+      </c>
+      <c r="M2">
+        <v>0.05</v>
+      </c>
+      <c r="N2">
+        <v>0</v>
+      </c>
+      <c r="O2">
+        <v>0</v>
+      </c>
+      <c r="P2">
+        <v>0</v>
+      </c>
+      <c r="Q2">
+        <v>0</v>
+      </c>
+      <c r="R2">
         <v>90</v>
-      </c>
-      <c r="D2">
-        <v>28</v>
-      </c>
-      <c r="E2">
-        <v>0.8</v>
-      </c>
-      <c r="F2" t="str">
-        <v>230,70,70</v>
-      </c>
-      <c r="G2">
-        <v>120</v>
-      </c>
-      <c r="H2">
-        <v>18</v>
-      </c>
-      <c r="I2">
-        <v>4</v>
-      </c>
-      <c r="J2">
-        <v>0</v>
-      </c>
-      <c r="K2">
-        <v>1</v>
-      </c>
-      <c r="L2">
-        <v>0.05</v>
-      </c>
-      <c r="M2">
-        <v>0.5</v>
-      </c>
-      <c r="N2">
-        <v>0.05</v>
-      </c>
-      <c r="O2">
-        <v>0</v>
-      </c>
-      <c r="P2">
-        <v>0</v>
-      </c>
-      <c r="Q2">
-        <v>0</v>
-      </c>
-      <c r="R2">
-        <v>0</v>
       </c>
       <c r="S2">
         <v>5</v>
@@ -705,52 +717,52 @@
         <v>疾行者</v>
       </c>
       <c r="C3">
+        <v>22</v>
+      </c>
+      <c r="D3">
+        <v>0.6</v>
+      </c>
+      <c r="E3" t="str">
+        <v>240,150,60</v>
+      </c>
+      <c r="F3">
+        <v>70</v>
+      </c>
+      <c r="G3">
+        <v>14</v>
+      </c>
+      <c r="H3">
+        <v>2</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <v>1.4</v>
+      </c>
+      <c r="K3">
+        <v>0.05</v>
+      </c>
+      <c r="L3">
+        <v>0.5</v>
+      </c>
+      <c r="M3">
+        <v>0.15</v>
+      </c>
+      <c r="N3">
+        <v>0</v>
+      </c>
+      <c r="O3">
+        <v>0</v>
+      </c>
+      <c r="P3">
+        <v>0</v>
+      </c>
+      <c r="Q3">
+        <v>0</v>
+      </c>
+      <c r="R3">
         <v>175</v>
-      </c>
-      <c r="D3">
-        <v>22</v>
-      </c>
-      <c r="E3">
-        <v>0.6</v>
-      </c>
-      <c r="F3" t="str">
-        <v>240,150,60</v>
-      </c>
-      <c r="G3">
-        <v>70</v>
-      </c>
-      <c r="H3">
-        <v>14</v>
-      </c>
-      <c r="I3">
-        <v>2</v>
-      </c>
-      <c r="J3">
-        <v>0</v>
-      </c>
-      <c r="K3">
-        <v>1.4</v>
-      </c>
-      <c r="L3">
-        <v>0.05</v>
-      </c>
-      <c r="M3">
-        <v>0.5</v>
-      </c>
-      <c r="N3">
-        <v>0.15</v>
-      </c>
-      <c r="O3">
-        <v>0</v>
-      </c>
-      <c r="P3">
-        <v>0</v>
-      </c>
-      <c r="Q3">
-        <v>0</v>
-      </c>
-      <c r="R3">
-        <v>0</v>
       </c>
       <c r="S3">
         <v>4</v>
@@ -764,52 +776,52 @@
         <v>重装</v>
       </c>
       <c r="C4">
+        <v>40</v>
+      </c>
+      <c r="D4">
+        <v>1.2</v>
+      </c>
+      <c r="E4" t="str">
+        <v>170,80,200</v>
+      </c>
+      <c r="F4">
+        <v>360</v>
+      </c>
+      <c r="G4">
+        <v>30</v>
+      </c>
+      <c r="H4">
+        <v>12</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>0.8</v>
+      </c>
+      <c r="K4">
+        <v>0.05</v>
+      </c>
+      <c r="L4">
+        <v>0.5</v>
+      </c>
+      <c r="M4">
+        <v>0</v>
+      </c>
+      <c r="N4">
+        <v>0</v>
+      </c>
+      <c r="O4">
+        <v>0</v>
+      </c>
+      <c r="P4">
+        <v>0</v>
+      </c>
+      <c r="Q4">
+        <v>0.15</v>
+      </c>
+      <c r="R4">
         <v>55</v>
-      </c>
-      <c r="D4">
-        <v>40</v>
-      </c>
-      <c r="E4">
-        <v>1.2</v>
-      </c>
-      <c r="F4" t="str">
-        <v>170,80,200</v>
-      </c>
-      <c r="G4">
-        <v>360</v>
-      </c>
-      <c r="H4">
-        <v>30</v>
-      </c>
-      <c r="I4">
-        <v>12</v>
-      </c>
-      <c r="J4">
-        <v>0</v>
-      </c>
-      <c r="K4">
-        <v>0.8</v>
-      </c>
-      <c r="L4">
-        <v>0.05</v>
-      </c>
-      <c r="M4">
-        <v>0.5</v>
-      </c>
-      <c r="N4">
-        <v>0</v>
-      </c>
-      <c r="O4">
-        <v>0</v>
-      </c>
-      <c r="P4">
-        <v>0</v>
-      </c>
-      <c r="Q4">
-        <v>0</v>
-      </c>
-      <c r="R4">
-        <v>0.15</v>
       </c>
       <c r="S4">
         <v>10</v>
@@ -823,52 +835,52 @@
         <v>屠夫领主</v>
       </c>
       <c r="C5">
+        <v>60</v>
+      </c>
+      <c r="D5">
+        <v>1.5</v>
+      </c>
+      <c r="E5" t="str">
+        <v>150,40,40</v>
+      </c>
+      <c r="F5">
+        <v>15100</v>
+      </c>
+      <c r="G5">
+        <v>55</v>
+      </c>
+      <c r="H5">
+        <v>20</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>0.8</v>
+      </c>
+      <c r="K5">
+        <v>0.05</v>
+      </c>
+      <c r="L5">
+        <v>0.5</v>
+      </c>
+      <c r="M5">
+        <v>0</v>
+      </c>
+      <c r="N5">
+        <v>0</v>
+      </c>
+      <c r="O5">
+        <v>0</v>
+      </c>
+      <c r="P5">
+        <v>0</v>
+      </c>
+      <c r="Q5">
+        <v>0.3</v>
+      </c>
+      <c r="R5">
         <v>40</v>
-      </c>
-      <c r="D5">
-        <v>60</v>
-      </c>
-      <c r="E5">
-        <v>1.5</v>
-      </c>
-      <c r="F5" t="str">
-        <v>150,40,40</v>
-      </c>
-      <c r="G5">
-        <v>15100</v>
-      </c>
-      <c r="H5">
-        <v>55</v>
-      </c>
-      <c r="I5">
-        <v>20</v>
-      </c>
-      <c r="J5">
-        <v>0</v>
-      </c>
-      <c r="K5">
-        <v>0.8</v>
-      </c>
-      <c r="L5">
-        <v>0.05</v>
-      </c>
-      <c r="M5">
-        <v>0.5</v>
-      </c>
-      <c r="N5">
-        <v>0</v>
-      </c>
-      <c r="O5">
-        <v>0</v>
-      </c>
-      <c r="P5">
-        <v>0</v>
-      </c>
-      <c r="Q5">
-        <v>0</v>
-      </c>
-      <c r="R5">
-        <v>0.3</v>
       </c>
       <c r="S5">
         <v>200</v>
@@ -883,7 +895,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:F4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -896,15 +908,12 @@
         <v>fireInterval</v>
       </c>
       <c r="D1" t="str">
-        <v>moveSpeed</v>
+        <v>advanceLimit</v>
       </c>
       <c r="E1" t="str">
-        <v>advanceLimit</v>
+        <v>healPerSec</v>
       </c>
       <c r="F1" t="str">
-        <v>healPerSec</v>
-      </c>
-      <c r="G1" t="str">
         <v>size</v>
       </c>
     </row>
@@ -919,15 +928,12 @@
         <v>0.5</v>
       </c>
       <c r="D2">
-        <v>300</v>
+        <v>80</v>
       </c>
       <c r="E2">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="F2">
-        <v>0</v>
-      </c>
-      <c r="G2">
         <v>74</v>
       </c>
     </row>
@@ -942,15 +948,12 @@
         <v>0.33</v>
       </c>
       <c r="D3">
-        <v>300</v>
+        <v>80</v>
       </c>
       <c r="E3">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="F3">
-        <v>0</v>
-      </c>
-      <c r="G3">
         <v>52</v>
       </c>
     </row>
@@ -968,18 +971,15 @@
         <v>0</v>
       </c>
       <c r="E4">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="F4">
-        <v>16</v>
-      </c>
-      <c r="G4">
         <v>52</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F4"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
balance(关卡): 技能 2 槽制 pacing 重校——L3 减负/L7 覆盖 -5%/L10 Boss 39000
- 根因（50 局诊断实证）：dps 移除 timer 型 ground_smash 后裸装档输出结构变化，L3 裸装真实胜率跌至 84%
- L3 减负至 96%、L7 4~6段 100% 过且 1~3段 0% 卡、L10 对冲坚壁被动恢复卡关余量
- 全量 13 门槛六连跑全绿；诊断口径与数值理由留档种子注释

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/config-xlsx/battle.xlsx
+++ b/tools/config-xlsx/battle.xlsx
@@ -1385,13 +1385,13 @@
         <v>zombie</v>
       </c>
       <c r="G14">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="H14">
         <v>0.4</v>
       </c>
       <c r="I14">
-        <v>150</v>
+        <v>110</v>
       </c>
     </row>
     <row r="15">
@@ -1414,7 +1414,7 @@
         <v>runner</v>
       </c>
       <c r="G15">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H15">
         <v>1</v>
@@ -1443,7 +1443,7 @@
         <v>brute</v>
       </c>
       <c r="G16">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H16">
         <v>1.5</v>
@@ -1472,7 +1472,7 @@
         <v>zombie</v>
       </c>
       <c r="G17">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H17">
         <v>0.4</v>
@@ -2058,7 +2058,7 @@
         <v>0.4</v>
       </c>
       <c r="I37">
-        <v>770</v>
+        <v>730</v>
       </c>
     </row>
     <row r="38">
@@ -2087,7 +2087,7 @@
         <v>1.2</v>
       </c>
       <c r="I38">
-        <v>2168</v>
+        <v>2060</v>
       </c>
     </row>
     <row r="39">
@@ -2116,7 +2116,7 @@
         <v>0.4</v>
       </c>
       <c r="I39">
-        <v>426</v>
+        <v>405</v>
       </c>
     </row>
     <row r="40">
@@ -2145,7 +2145,7 @@
         <v>1.2</v>
       </c>
       <c r="I40">
-        <v>2168</v>
+        <v>2060</v>
       </c>
     </row>
     <row r="41">
@@ -2174,7 +2174,7 @@
         <v>0.4</v>
       </c>
       <c r="I41">
-        <v>770</v>
+        <v>730</v>
       </c>
     </row>
     <row r="42">
@@ -2203,7 +2203,7 @@
         <v>1.4</v>
       </c>
       <c r="I42">
-        <v>2168</v>
+        <v>2060</v>
       </c>
     </row>
     <row r="43">
@@ -2232,7 +2232,7 @@
         <v>0.6</v>
       </c>
       <c r="I43">
-        <v>426</v>
+        <v>405</v>
       </c>
     </row>
     <row r="44">
@@ -2812,7 +2812,7 @@
         <v>1</v>
       </c>
       <c r="I63">
-        <v>36000</v>
+        <v>39000</v>
       </c>
     </row>
     <row r="64">

</xml_diff>